<commit_message>
feat: Add visualization utilities and integrate into main workflow
- Created a new module `utils.py` for auxiliary functions related to visualizations, including date extraction, formatting, and color scale generation.
- Updated `main.py` to include visualization generation after optimization, with error handling for missing visualization module.
- Introduced a new function `calcular_estadisticas_correctas` to compute corrected statistics from optimization results.
- Added a new option in the menu for generating only visualizations.
- Updated requirements to include `plotly` and `kaleido` for enhanced visualization capabilities.
- Created a new `visualizaciones.py` module to maintain compatibility with the main application while redirecting to improved visualization functions.
</commit_message>
<xml_diff>
--- a/output/estadisticas_ofertas.xlsx
+++ b/output/estadisticas_ofertas.xlsx
@@ -463,17 +463,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OP1_Wide -AES</t>
+          <t>OP1_Wide- EPM</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>415000000.0000029</v>
+        <v>916608868</v>
       </c>
       <c r="D2" t="n">
-        <v>129.5714928739288</v>
+        <v>55.94211962701859</v>
       </c>
       <c r="E2" t="n">
-        <v>53772169542.68082</v>
+        <v>51277042944.84209</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +484,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OP1_Wide -ISAGEN</t>
+          <t>OP1_Wide -AES</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>459458287.0000031</v>
+        <v>415000000.0000029</v>
       </c>
       <c r="D3" t="n">
-        <v>81.67845026912242</v>
+        <v>129.5714928739288</v>
       </c>
       <c r="E3" t="n">
-        <v>37527840845.46593</v>
+        <v>53772169542.68082</v>
       </c>
     </row>
     <row r="4">
@@ -505,17 +505,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OP1_Wide- EPM</t>
+          <t>OP1_Wide -ISAGEN</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>880608868</v>
+        <v>423458287.0000017</v>
       </c>
       <c r="D4" t="n">
-        <v>53.76483966340702</v>
+        <v>81.67845026912254</v>
       </c>
       <c r="E4" t="n">
-        <v>47345794594.19435</v>
+        <v>34587416635.77745</v>
       </c>
     </row>
     <row r="5">
@@ -530,13 +530,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1755067155.000006</v>
+        <v>1755067155.000005</v>
       </c>
       <c r="D5" t="n">
-        <v>78.9974358458897</v>
+        <v>79.56198640347753</v>
       </c>
       <c r="E5" t="n">
-        <v>138645804982.3411</v>
+        <v>139636629123.3004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implementa un validador de nombres de ofertas con formato estandarizado en core/validador_ofertas.py.
</commit_message>
<xml_diff>
--- a/output/estadisticas_ofertas.xlsx
+++ b/output/estadisticas_ofertas.xlsx
@@ -463,7 +463,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OP1_Wide -AES</t>
+          <t>AES-OFERTA-001</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -484,17 +484,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OP1_Wide -ISAGEN</t>
+          <t>EPM-OFERTA-001</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>423458287.0000017</v>
+        <v>916608868</v>
       </c>
       <c r="D3" t="n">
-        <v>81.67845026912254</v>
+        <v>55.94211962701859</v>
       </c>
       <c r="E3" t="n">
-        <v>34587416635.77745</v>
+        <v>51277042944.84209</v>
       </c>
     </row>
     <row r="4">
@@ -505,17 +505,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OP1_Wide- EPM</t>
+          <t>ISAGEN-OFERTA-001</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>916608868</v>
+        <v>423458287.0000017</v>
       </c>
       <c r="D4" t="n">
-        <v>55.94211962701859</v>
+        <v>81.67845026912254</v>
       </c>
       <c r="E4" t="n">
-        <v>51277042944.84209</v>
+        <v>34587416635.77745</v>
       </c>
     </row>
     <row r="5">
@@ -533,7 +533,7 @@
         <v>1755067155.000005</v>
       </c>
       <c r="D5" t="n">
-        <v>79.56198640347755</v>
+        <v>79.56198640347753</v>
       </c>
       <c r="E5" t="n">
         <v>139636629123.3004</v>

</xml_diff>

<commit_message>
Correcciones de las grafiacas 5,6,7 se agrago el  mw_promedio
</commit_message>
<xml_diff>
--- a/output/estadisticas_ofertas.xlsx
+++ b/output/estadisticas_ofertas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,13 +467,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>415000000.0000029</v>
+        <v>46128910.32313082</v>
       </c>
       <c r="D2" t="n">
-        <v>129.5714928739288</v>
+        <v>48.69033525265036</v>
       </c>
       <c r="E2" t="n">
-        <v>53772169542.68082</v>
+        <v>2246032108.472683</v>
       </c>
     </row>
     <row r="3">
@@ -484,17 +484,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EPM-OFERTA-001</t>
+          <t>AMPERIA-OFERTA-001</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>916608868</v>
+        <v>21896000</v>
       </c>
       <c r="D3" t="n">
-        <v>55.94211962701859</v>
+        <v>55.28610464137377</v>
       </c>
       <c r="E3" t="n">
-        <v>51277042944.84209</v>
+        <v>1210544547.22752</v>
       </c>
     </row>
     <row r="4">
@@ -505,38 +505,332 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ISAGEN-OFERTA-001</t>
+          <t>BTG-OFERTA-001</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>423458287.0000017</v>
+        <v>1574933.751241006</v>
       </c>
       <c r="D4" t="n">
-        <v>81.67845026912254</v>
+        <v>10.47044260307196</v>
       </c>
       <c r="E4" t="n">
-        <v>34587416635.77745</v>
+        <v>16490253.44600976</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BTG-OFERTA-003</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>6616365.521153433</v>
+      </c>
+      <c r="D5" t="n">
+        <v>22.76253031527892</v>
+      </c>
+      <c r="E5" t="n">
+        <v>150605220.7522212</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BTG-OFERTA-006</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>620000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9.190430476960387</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5698066.89571544</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BTG-OFERTA-007</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10661461.351379</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9.813510509296579</v>
+      </c>
+      <c r="E7" t="n">
+        <v>104626363.0162171</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BTG-OFERTA-008</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8000509.411154016</v>
+      </c>
+      <c r="D8" t="n">
+        <v>10.12505052546483</v>
+      </c>
+      <c r="E8" t="n">
+        <v>81005562.01739132</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BTG-OFERTA-009</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>620000</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10.43659054163298</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6470686.13581245</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DEPIENERGY-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>7164021.976300159</v>
+      </c>
+      <c r="D10" t="n">
+        <v>61.42928119105346</v>
+      </c>
+      <c r="E10" t="n">
+        <v>440080720.441029</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DICELER-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2625000</v>
+      </c>
+      <c r="D11" t="n">
+        <v>21.78122309368781</v>
+      </c>
+      <c r="E11" t="n">
+        <v>57175710.62093049</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DICELER-OFERTA-002</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1289122.927112857</v>
+      </c>
+      <c r="D12" t="n">
+        <v>22.41256289350486</v>
+      </c>
+      <c r="E12" t="n">
+        <v>28892548.68137598</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ISAGEN-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>102999999.77</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PROENERGY-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7651505.04724499</v>
+      </c>
+      <c r="D14" t="n">
+        <v>41.13772500403599</v>
+      </c>
+      <c r="E14" t="n">
+        <v>314765510.5005578</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PUTUMAYO-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>8485943.33029063</v>
+      </c>
+      <c r="D15" t="n">
+        <v>40.70523443815681</v>
+      </c>
+      <c r="E15" t="n">
+        <v>345422312.6883932</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PUTUMAYO-OFERTA-002</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2999999.99999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>12.19179466451092</v>
+      </c>
+      <c r="E16" t="n">
+        <v>36575383.99353264</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PUTUMAYO-OFERTA-003</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>15179141.85480185</v>
+      </c>
+      <c r="D17" t="n">
+        <v>28.16902452169227</v>
+      </c>
+      <c r="E17" t="n">
+        <v>427581619.1261588</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>OFERTA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>VATIA-OFERTA-001</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>15473257.84837405</v>
+      </c>
+      <c r="D18" t="n">
+        <v>28.38801872810563</v>
+      </c>
+      <c r="E18" t="n">
+        <v>439255133.5844499</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>TODAS LAS OFERTAS</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>1755067155.000005</v>
-      </c>
-      <c r="D5" t="n">
-        <v>79.56198640347753</v>
-      </c>
-      <c r="E5" t="n">
-        <v>139636629123.3004</v>
+      <c r="C19" t="n">
+        <v>259986173.1121828</v>
+      </c>
+      <c r="D19" t="n">
+        <v>22.73667740418385</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5911221747.599998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>